<commit_message>
Strengthen bird GEB-style effort analysis robustness
</commit_message>
<xml_diff>
--- a/tasks/bird_geb_fig3_fig4_effort_analysis/results/bird_geb_fig3_fig4_analysis_bundle.xlsx
+++ b/tasks/bird_geb_fig3_fig4_effort_analysis/results/bird_geb_fig3_fig4_analysis_bundle.xlsx
@@ -12,10 +12,15 @@
     <sheet name="effort_coverage_by_province" sheetId="3" r:id="rId3"/>
     <sheet name="species_coefficients" sheetId="4" r:id="rId4"/>
     <sheet name="province_coefficients" sheetId="5" r:id="rId5"/>
-    <sheet name="province_sensitivity" sheetId="6" r:id="rId6"/>
-    <sheet name="province_importance" sheetId="7" r:id="rId7"/>
-    <sheet name="province_importance_boot_ci" sheetId="8" r:id="rId8"/>
-    <sheet name="province_diagnostics" sheetId="9" r:id="rId9"/>
+    <sheet name="province_user_effort_coeffici" sheetId="6" r:id="rId6"/>
+    <sheet name="province_sensitivity" sheetId="7" r:id="rId7"/>
+    <sheet name="province_influence_coefficien" sheetId="8" r:id="rId8"/>
+    <sheet name="province_importance" sheetId="9" r:id="rId9"/>
+    <sheet name="province_importance_boot_ci" sheetId="10" r:id="rId10"/>
+    <sheet name="province_diagnostics" sheetId="11" r:id="rId11"/>
+    <sheet name="province_model_comparison" sheetId="12" r:id="rId12"/>
+    <sheet name="province_influential_units" sheetId="13" r:id="rId13"/>
+    <sheet name="predictor_source_audit" sheetId="14" r:id="rId14"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -459,6 +464,993 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>term</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>predictor</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>independent_r2_mean</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>independent_r2_low</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>independent_r2_high</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>percent_mean</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>percent_low</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>percent_high</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>z_area_km2</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>0.3159625221796286</v>
+      </c>
+      <c r="D2">
+        <v>0.1774893787662221</v>
+      </c>
+      <c r="E2">
+        <v>0.496176654019657</v>
+      </c>
+      <c r="F2">
+        <v>46.3885174002197</v>
+      </c>
+      <c r="G2">
+        <v>24.492743670897</v>
+      </c>
+      <c r="H2">
+        <v>75.15963261531341</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>z_curr_report_density</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Current survey effort</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>0.1906731864260424</v>
+      </c>
+      <c r="D3">
+        <v>0.0610965322137838</v>
+      </c>
+      <c r="E3">
+        <v>0.3478016293982022</v>
+      </c>
+      <c r="F3">
+        <v>27.24958641333323</v>
+      </c>
+      <c r="G3">
+        <v>9.767496958990433</v>
+      </c>
+      <c r="H3">
+        <v>46.55143366824811</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>z_gdp_per_capita</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Per capita GDP</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>0.1414321566113755</v>
+      </c>
+      <c r="D4">
+        <v>0.02465196908661925</v>
+      </c>
+      <c r="E4">
+        <v>0.2627245599856989</v>
+      </c>
+      <c r="F4">
+        <v>20.41835047307</v>
+      </c>
+      <c r="G4">
+        <v>3.951531585325443</v>
+      </c>
+      <c r="H4">
+        <v>35.56228432739437</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>z_habitat_heterogeneity</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Habitat heterogeneity</t>
+        </is>
+      </c>
+      <c r="C5">
+        <v>0.02156300811270996</v>
+      </c>
+      <c r="D5">
+        <v>0.002258926997642939</v>
+      </c>
+      <c r="E5">
+        <v>0.07717711991280371</v>
+      </c>
+      <c r="F5">
+        <v>3.183483636623861</v>
+      </c>
+      <c r="G5">
+        <v>0.3358428395250163</v>
+      </c>
+      <c r="H5">
+        <v>11.15504161120841</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>z_hist_report_density</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Historical survey effort</t>
+        </is>
+      </c>
+      <c r="C6">
+        <v>0.01851734543026135</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>0.06619297387946545</v>
+      </c>
+      <c r="F6">
+        <v>2.760062076753207</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>10.17575527515512</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>n_provinces_modelled</t>
+        </is>
+      </c>
+      <c r="B2">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>adjusted_r2_primary</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>0.6532642079775428</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>shapiro_p_residuals</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>0.0951965390723178</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ncvtest_p_heteroskedasticity</t>
+        </is>
+      </c>
+      <c r="B5">
+        <v>0.5118818185685223</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>max_cooks_distance</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>128.333766474755</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>overdispersion_ratio_sensitivity</t>
+        </is>
+      </c>
+      <c r="B7">
+        <v>1.006653737424887</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>n_influential_provinces</t>
+        </is>
+      </c>
+      <c r="B8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>influence_threshold_4_over_n</t>
+        </is>
+      </c>
+      <c r="B9">
+        <v>0.1290322580645161</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>aic</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>bic</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>r_squared</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>adj_r_squared</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>max_vif</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Primary report-effort model</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Gaussian LM</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>68.29227619531429</v>
+      </c>
+      <c r="D2">
+        <v>78.33018662671032</v>
+      </c>
+      <c r="E2">
+        <v>0.7110535066479523</v>
+      </c>
+      <c r="F2">
+        <v>0.6532642079775428</v>
+      </c>
+      <c r="G2">
+        <v>2.98687299639897</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Alternative user-effort model</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Gaussian LM</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>67.18722389882413</v>
+      </c>
+      <c r="D3">
+        <v>77.22513433022016</v>
+      </c>
+      <c r="E3">
+        <v>0.7211721186895074</v>
+      </c>
+      <c r="F3">
+        <v>0.6654065424274089</v>
+      </c>
+      <c r="G3">
+        <v>3.033311466595738</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Influence-filtered report-effort model</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Gaussian LM</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>53.20262951069085</v>
+      </c>
+      <c r="D4">
+        <v>62.77370032059616</v>
+      </c>
+      <c r="E4">
+        <v>0.7766436813927878</v>
+      </c>
+      <c r="F4">
+        <v>0.7280879599564374</v>
+      </c>
+      <c r="G4">
+        <v>2.993128252086424</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Count-based sensitivity model</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Negative binomial</t>
+        </is>
+      </c>
+      <c r="C5">
+        <v>305.9627043913289</v>
+      </c>
+      <c r="D5">
+        <v>314.5666276182398</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:AI3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>province</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>n_records</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>n_species</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>current_report_sum</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>historical_report_sum</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>current_user_sum</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>historical_user_sum</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>historical_report_annual</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>current_report_annual</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>historical_user_annual</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>current_user_annual</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>gdp_per_capita</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>area_km2</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>habitat_heterogeneity</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>human_density</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>population_10k</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>reference_mammal_richness</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>new_record_density_100k</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>log_new_record_density</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>historical_report_density</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>current_report_density</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>historical_user_density</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>current_user_density</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>z_hist_report_density</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>z_curr_report_density</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>z_gdp_per_capita</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>z_area_km2</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>z_habitat_heterogeneity</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>z_curr_user_density</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>fitted_primary</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>resid_primary</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>std_resid_primary</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>cooks_d_primary</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>hat_primary</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>dffits_primary</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Jiangsu</t>
+        </is>
+      </c>
+      <c r="B2">
+        <v>50</v>
+      </c>
+      <c r="C2">
+        <v>50</v>
+      </c>
+      <c r="D2">
+        <v>47456</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
+      </c>
+      <c r="F2">
+        <v>4796</v>
+      </c>
+      <c r="G2">
+        <v>3</v>
+      </c>
+      <c r="H2">
+        <v>0.25</v>
+      </c>
+      <c r="I2">
+        <v>1898.24</v>
+      </c>
+      <c r="J2">
+        <v>0.15</v>
+      </c>
+      <c r="K2">
+        <v>191.84</v>
+      </c>
+      <c r="L2">
+        <v>144989</v>
+      </c>
+      <c r="M2">
+        <v>107200</v>
+      </c>
+      <c r="N2">
+        <v>1.336322</v>
+      </c>
+      <c r="O2">
+        <v>791</v>
+      </c>
+      <c r="P2">
+        <v>8475</v>
+      </c>
+      <c r="Q2">
+        <v>62</v>
+      </c>
+      <c r="R2">
+        <v>46.64179104477612</v>
+      </c>
+      <c r="S2">
+        <v>3.863710339178733</v>
+      </c>
+      <c r="T2">
+        <v>0.2332089552238806</v>
+      </c>
+      <c r="U2">
+        <v>1770.746268656716</v>
+      </c>
+      <c r="V2">
+        <v>0.1399253731343283</v>
+      </c>
+      <c r="W2">
+        <v>178.955223880597</v>
+      </c>
+      <c r="X2">
+        <v>5.384875299116219</v>
+      </c>
+      <c r="Y2">
+        <v>-0.09549536202885804</v>
+      </c>
+      <c r="Z2">
+        <v>1.671236711133321</v>
+      </c>
+      <c r="AA2">
+        <v>-0.5255944978764049</v>
+      </c>
+      <c r="AB2">
+        <v>-1.01204021865528</v>
+      </c>
+      <c r="AC2">
+        <v>-0.05447143178517364</v>
+      </c>
+      <c r="AD2">
+        <v>3.880366460202694</v>
+      </c>
+      <c r="AE2">
+        <v>-0.01665612102396051</v>
+      </c>
+      <c r="AF2">
+        <v>-0.8455163339356818</v>
+      </c>
+      <c r="AG2">
+        <v>128.333766474755</v>
+      </c>
+      <c r="AH2">
+        <v>0.999072425533357</v>
+      </c>
+      <c r="AI2">
+        <v>-27.58555647289191</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tianjin</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>26</v>
+      </c>
+      <c r="C3">
+        <v>25</v>
+      </c>
+      <c r="D3">
+        <v>9815</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>1055</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>392.6</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>42.2</v>
+      </c>
+      <c r="L3">
+        <v>117635</v>
+      </c>
+      <c r="M3">
+        <v>11934</v>
+      </c>
+      <c r="N3">
+        <v>1.3320304</v>
+      </c>
+      <c r="O3">
+        <v>1162</v>
+      </c>
+      <c r="P3">
+        <v>1387</v>
+      </c>
+      <c r="Q3">
+        <v>22</v>
+      </c>
+      <c r="R3">
+        <v>217.8649237472767</v>
+      </c>
+      <c r="S3">
+        <v>5.388454752983316</v>
+      </c>
+      <c r="T3">
+        <v>0</v>
+      </c>
+      <c r="U3">
+        <v>3289.760348583878</v>
+      </c>
+      <c r="V3">
+        <v>0</v>
+      </c>
+      <c r="W3">
+        <v>353.6115300821183</v>
+      </c>
+      <c r="X3">
+        <v>-0.1859779388983075</v>
+      </c>
+      <c r="Y3">
+        <v>0.09349206279565123</v>
+      </c>
+      <c r="Z3">
+        <v>0.9156267998356485</v>
+      </c>
+      <c r="AA3">
+        <v>-0.7712966914337204</v>
+      </c>
+      <c r="AB3">
+        <v>-1.024777585556462</v>
+      </c>
+      <c r="AC3">
+        <v>0.2434445904125866</v>
+      </c>
+      <c r="AD3">
+        <v>3.656961983311166</v>
+      </c>
+      <c r="AE3">
+        <v>1.73149276967215</v>
+      </c>
+      <c r="AF3">
+        <v>2.956916293242752</v>
+      </c>
+      <c r="AG3">
+        <v>0.3207198741604326</v>
+      </c>
+      <c r="AH3">
+        <v>0.1803879071887361</v>
+      </c>
+      <c r="AI3">
+        <v>1.685499808915389</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>variable</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>source_file</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>used_in_primary_bird_model</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>rationale</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>gdp_per_capita</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Province_variables.csv</t>
+        </is>
+      </c>
+      <c r="C2" t="b">
+        <v>1</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Generic socioeconomic covariate transferable across taxa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>area_km2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Province_variables.csv</t>
+        </is>
+      </c>
+      <c r="C3" t="b">
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Generic geographic covariate transferable across taxa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>habitat_heterogeneity</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Province_variables.csv</t>
+        </is>
+      </c>
+      <c r="C4" t="b">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Generic environmental heterogeneity covariate transferable across taxa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>human_density</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Province_variables.csv</t>
+        </is>
+      </c>
+      <c r="C5" t="b">
+        <v>0</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Screened only; not retained because current user effort was already available directly and highly collinear with current report effort.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>reference_mammal_richness</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Province_variables.csv</t>
+        </is>
+      </c>
+      <c r="C6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Not used because this richness field originates from the mammal GEB workflow and is therefore taxonomically mismatched for a bird-specific model.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C6"/>
@@ -2258,7 +3250,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -2310,22 +3302,22 @@
         </is>
       </c>
       <c r="B2">
-        <v>-0.07038901351962511</v>
+        <v>0.07351518884548884</v>
       </c>
       <c r="C2">
-        <v>0.1719406119586797</v>
+        <v>0.1359377234840907</v>
       </c>
       <c r="D2">
-        <v>-0.4093798010707371</v>
+        <v>0.5408005001208704</v>
       </c>
       <c r="E2">
-        <v>0.6822609605523682</v>
+        <v>0.593431430140716</v>
       </c>
       <c r="F2">
-        <v>-0.4073926129586374</v>
+        <v>-0.1929227491833289</v>
       </c>
       <c r="G2">
-        <v>0.2666145859193871</v>
+        <v>0.3399531268743066</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -2336,30 +3328,30 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>z_curr_report_density</t>
+          <t>z_curr_user_density</t>
         </is>
       </c>
       <c r="B3">
-        <v>0.2581832009469735</v>
+        <v>0.4923900703287938</v>
       </c>
       <c r="C3">
-        <v>0.2453606689374848</v>
+        <v>0.1951994978788663</v>
       </c>
       <c r="D3">
-        <v>1.052259932551601</v>
+        <v>2.522496603112951</v>
       </c>
       <c r="E3">
-        <v>0.2926803091743495</v>
+        <v>0.01838869401193881</v>
       </c>
       <c r="F3">
-        <v>-0.2227237101704967</v>
+        <v>0.109799054486216</v>
       </c>
       <c r="G3">
-        <v>0.7390901120644437</v>
+        <v>0.8749810861713717</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Current survey effort</t>
+          <t>Current user effort</t>
         </is>
       </c>
     </row>
@@ -2370,22 +3362,22 @@
         </is>
       </c>
       <c r="B4">
-        <v>0.5125644436099142</v>
+        <v>0.1020835537928959</v>
       </c>
       <c r="C4">
-        <v>0.2514191185196972</v>
+        <v>0.2020387787008036</v>
       </c>
       <c r="D4">
-        <v>2.038685230573496</v>
+        <v>0.5052671296537088</v>
       </c>
       <c r="E4">
-        <v>0.04148145273116593</v>
+        <v>0.6177968537907309</v>
       </c>
       <c r="F4">
-        <v>0.01978297131130757</v>
+        <v>-0.2939124524606792</v>
       </c>
       <c r="G4">
-        <v>1.005345915908521</v>
+        <v>0.498079560046471</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -2396,28 +3388,58 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>z_area_km2</t>
+        </is>
+      </c>
+      <c r="B5">
+        <v>-0.5784447440021174</v>
+      </c>
+      <c r="C5">
+        <v>0.1220030873557291</v>
+      </c>
+      <c r="D5">
+        <v>-4.741230378174969</v>
+      </c>
+      <c r="E5">
+        <v>7.286192370789932E-05</v>
+      </c>
+      <c r="F5">
+        <v>-0.8175707952193465</v>
+      </c>
+      <c r="G5">
+        <v>-0.3393186927848884</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>z_habitat_heterogeneity</t>
         </is>
       </c>
-      <c r="B5">
-        <v>-0.1222295065390467</v>
-      </c>
-      <c r="C5">
-        <v>0.1553235780359703</v>
-      </c>
-      <c r="D5">
-        <v>-0.7869346565705594</v>
-      </c>
-      <c r="E5">
-        <v>0.4313201185768374</v>
-      </c>
-      <c r="F5">
-        <v>-0.4266637194895485</v>
-      </c>
-      <c r="G5">
-        <v>0.182204706411455</v>
-      </c>
-      <c r="H5" t="inlineStr">
+      <c r="B6">
+        <v>-0.03664674305324695</v>
+      </c>
+      <c r="C6">
+        <v>0.123320476562611</v>
+      </c>
+      <c r="D6">
+        <v>-0.2971667323604694</v>
+      </c>
+      <c r="E6">
+        <v>0.768794412703406</v>
+      </c>
+      <c r="F6">
+        <v>-0.2783548771159644</v>
+      </c>
+      <c r="G6">
+        <v>0.2050613910094705</v>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>Habitat heterogeneity</t>
         </is>
@@ -2430,7 +3452,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -2441,15 +3463,35 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>independent_r2</t>
+          <t>estimate</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>std.error</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>statistic</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>p.value</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>conf.low</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>conf.high</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>predictor</t>
         </is>
@@ -2462,12 +3504,24 @@
         </is>
       </c>
       <c r="B2">
-        <v>0.00816896007520326</v>
+        <v>-0.07038901351962511</v>
       </c>
       <c r="C2">
-        <v>1.228479355686827</v>
-      </c>
-      <c r="D2" t="inlineStr">
+        <v>0.1719406119586797</v>
+      </c>
+      <c r="D2">
+        <v>-0.4093798010707371</v>
+      </c>
+      <c r="E2">
+        <v>0.6822609605523682</v>
+      </c>
+      <c r="F2">
+        <v>-0.4073926129586374</v>
+      </c>
+      <c r="G2">
+        <v>0.2666145859193871</v>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>Historical survey effort</t>
         </is>
@@ -2480,12 +3534,24 @@
         </is>
       </c>
       <c r="B3">
-        <v>0.1890127849374196</v>
+        <v>0.2581832009469735</v>
       </c>
       <c r="C3">
-        <v>28.42446310410161</v>
-      </c>
-      <c r="D3" t="inlineStr">
+        <v>0.2453606689374848</v>
+      </c>
+      <c r="D3">
+        <v>1.052259932551601</v>
+      </c>
+      <c r="E3">
+        <v>0.2926803091743495</v>
+      </c>
+      <c r="F3">
+        <v>-0.2227237101704967</v>
+      </c>
+      <c r="G3">
+        <v>0.7390901120644437</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>Current survey effort</t>
         </is>
@@ -2498,12 +3564,24 @@
         </is>
       </c>
       <c r="B4">
-        <v>0.1441231711208185</v>
+        <v>0.5125644436099142</v>
       </c>
       <c r="C4">
-        <v>21.67379186189009</v>
-      </c>
-      <c r="D4" t="inlineStr">
+        <v>0.2514191185196972</v>
+      </c>
+      <c r="D4">
+        <v>2.038685230573496</v>
+      </c>
+      <c r="E4">
+        <v>0.04148145273116593</v>
+      </c>
+      <c r="F4">
+        <v>0.01978297131130757</v>
+      </c>
+      <c r="G4">
+        <v>1.005345915908521</v>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>Per capita GDP</t>
         </is>
@@ -2512,34 +3590,28 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>z_area_km2</t>
+          <t>z_habitat_heterogeneity</t>
         </is>
       </c>
       <c r="B5">
-        <v>0.3147448982106387</v>
+        <v>-0.1222295065390467</v>
       </c>
       <c r="C5">
-        <v>47.33253758127846</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Area</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>z_habitat_heterogeneity</t>
-        </is>
-      </c>
-      <c r="B6">
-        <v>0.008915375130845707</v>
-      </c>
-      <c r="C6">
-        <v>1.340728097043023</v>
-      </c>
-      <c r="D6" t="inlineStr">
+        <v>0.1553235780359703</v>
+      </c>
+      <c r="D5">
+        <v>-0.7869346565705594</v>
+      </c>
+      <c r="E5">
+        <v>0.4313201185768374</v>
+      </c>
+      <c r="F5">
+        <v>-0.4266637194895485</v>
+      </c>
+      <c r="G5">
+        <v>0.182204706411455</v>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>Habitat heterogeneity</t>
         </is>
@@ -2563,68 +3635,68 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>estimate</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>std.error</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>statistic</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>p.value</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>conf.low</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>conf.high</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>predictor</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>independent_r2_mean</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>independent_r2_low</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>independent_r2_high</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>percent_mean</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>percent_low</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>percent_high</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>z_area_km2</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Area</t>
-        </is>
+          <t>z_hist_report_density</t>
+        </is>
+      </c>
+      <c r="B2">
+        <v>3.041441327241234</v>
       </c>
       <c r="C2">
-        <v>0.3159625221796286</v>
+        <v>3.145562037650975</v>
       </c>
       <c r="D2">
-        <v>0.1774893787662221</v>
+        <v>0.9668991712248993</v>
       </c>
       <c r="E2">
-        <v>0.496176654019657</v>
+        <v>0.3436523110848047</v>
       </c>
       <c r="F2">
-        <v>46.3885174002197</v>
+        <v>-3.123860266554678</v>
       </c>
       <c r="G2">
-        <v>24.492743670897</v>
-      </c>
-      <c r="H2">
-        <v>75.15963261531341</v>
+        <v>9.206742921037145</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Historical survey effort</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -2633,28 +3705,28 @@
           <t>z_curr_report_density</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3">
+        <v>0.6069266275353788</v>
+      </c>
+      <c r="C3">
+        <v>0.1687610090485462</v>
+      </c>
+      <c r="D3">
+        <v>3.596367614516863</v>
+      </c>
+      <c r="E3">
+        <v>0.001523544253560398</v>
+      </c>
+      <c r="F3">
+        <v>0.2761550498002283</v>
+      </c>
+      <c r="G3">
+        <v>0.9376982052705294</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>Current survey effort</t>
         </is>
-      </c>
-      <c r="C3">
-        <v>0.1906731864260424</v>
-      </c>
-      <c r="D3">
-        <v>0.0610965322137838</v>
-      </c>
-      <c r="E3">
-        <v>0.3478016293982022</v>
-      </c>
-      <c r="F3">
-        <v>27.24958641333323</v>
-      </c>
-      <c r="G3">
-        <v>9.767496958990433</v>
-      </c>
-      <c r="H3">
-        <v>46.55143366824811</v>
       </c>
     </row>
     <row r="4">
@@ -2663,88 +3735,88 @@
           <t>z_gdp_per_capita</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4">
+        <v>-0.04382139894009667</v>
+      </c>
+      <c r="C4">
+        <v>0.1772708853651493</v>
+      </c>
+      <c r="D4">
+        <v>-0.2472002035180886</v>
+      </c>
+      <c r="E4">
+        <v>0.806946563583215</v>
+      </c>
+      <c r="F4">
+        <v>-0.3912723342557893</v>
+      </c>
+      <c r="G4">
+        <v>0.303629536375596</v>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>Per capita GDP</t>
         </is>
-      </c>
-      <c r="C4">
-        <v>0.1414321566113755</v>
-      </c>
-      <c r="D4">
-        <v>0.02465196908661925</v>
-      </c>
-      <c r="E4">
-        <v>0.2627245599856989</v>
-      </c>
-      <c r="F4">
-        <v>20.41835047307</v>
-      </c>
-      <c r="G4">
-        <v>3.951531585325443</v>
-      </c>
-      <c r="H4">
-        <v>35.56228432739437</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>z_habitat_heterogeneity</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Habitat heterogeneity</t>
-        </is>
+          <t>z_area_km2</t>
+        </is>
+      </c>
+      <c r="B5">
+        <v>-0.5911091780506049</v>
       </c>
       <c r="C5">
-        <v>0.02156300811270996</v>
+        <v>0.1138361508200725</v>
       </c>
       <c r="D5">
-        <v>0.002258926997642939</v>
+        <v>-5.192631460149266</v>
       </c>
       <c r="E5">
-        <v>0.07717711991280371</v>
+        <v>2.896414769927461E-05</v>
       </c>
       <c r="F5">
-        <v>3.183483636623861</v>
+        <v>-0.8142280336579469</v>
       </c>
       <c r="G5">
-        <v>0.3358428395250163</v>
-      </c>
-      <c r="H5">
-        <v>11.15504161120841</v>
+        <v>-0.3679903224432629</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>z_hist_report_density</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Historical survey effort</t>
-        </is>
+          <t>z_habitat_heterogeneity</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>0.06354516392940585</v>
       </c>
       <c r="C6">
-        <v>0.01851734543026135</v>
+        <v>0.1076008575905685</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>0.5905637311107804</v>
       </c>
       <c r="E6">
-        <v>0.06619297387946545</v>
+        <v>0.5605715079427503</v>
       </c>
       <c r="F6">
-        <v>2.760062076753207</v>
+        <v>-0.1473525169481083</v>
       </c>
       <c r="G6">
-        <v>0</v>
-      </c>
-      <c r="H6">
-        <v>10.17575527515512</v>
+        <v>0.27444284480692</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Habitat heterogeneity</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2754,79 +3826,119 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>metric</t>
+          <t>term</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>independent_r2</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>predictor</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>n_provinces_modelled</t>
+          <t>z_hist_report_density</t>
         </is>
       </c>
       <c r="B2">
-        <v>31</v>
+        <v>0.00816896007520326</v>
+      </c>
+      <c r="C2">
+        <v>1.228479355686827</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Historical survey effort</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>adjusted_r2_primary</t>
+          <t>z_curr_report_density</t>
         </is>
       </c>
       <c r="B3">
-        <v>0.6532642079775428</v>
+        <v>0.1890127849374196</v>
+      </c>
+      <c r="C3">
+        <v>28.42446310410161</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Current survey effort</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>shapiro_p_residuals</t>
+          <t>z_gdp_per_capita</t>
         </is>
       </c>
       <c r="B4">
-        <v>0.0951965390723178</v>
+        <v>0.1441231711208185</v>
+      </c>
+      <c r="C4">
+        <v>21.67379186189009</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Per capita GDP</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ncvtest_p_heteroskedasticity</t>
+          <t>z_area_km2</t>
         </is>
       </c>
       <c r="B5">
-        <v>0.5118818185685223</v>
+        <v>0.3147448982106387</v>
+      </c>
+      <c r="C5">
+        <v>47.33253758127846</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>max_cooks_distance</t>
+          <t>z_habitat_heterogeneity</t>
         </is>
       </c>
       <c r="B6">
-        <v>128.333766474755</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>overdispersion_ratio_sensitivity</t>
-        </is>
-      </c>
-      <c r="B7">
-        <v>1.006653737424887</v>
+        <v>0.008915375130845707</v>
+      </c>
+      <c r="C6">
+        <v>1.340728097043023</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Habitat heterogeneity</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>